<commit_message>
update to indicator list incl. HCAI sources and level of returns (provider or site)
</commit_message>
<xml_diff>
--- a/indicator_summary.xlsx
+++ b/indicator_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FB09759-1EED-457B-8AA7-73BCE596F62C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="58">
   <si>
     <t>id</t>
   </si>
@@ -101,9 +101,6 @@
     <t>Patient experience</t>
   </si>
   <si>
-    <t>Friends and Family test, UKHF</t>
-  </si>
-  <si>
     <t>Apr13 to Nov23</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
     <t>TBC</t>
   </si>
   <si>
-    <t>UKHSA TBC</t>
-  </si>
-  <si>
     <t>domain</t>
   </si>
   <si>
@@ -170,9 +164,6 @@
     <t>metric_reqd</t>
   </si>
   <si>
-    <t>number and rate per bed days</t>
-  </si>
-  <si>
     <t>number and rate per admission</t>
   </si>
   <si>
@@ -204,6 +195,21 @@
   </si>
   <si>
     <t>% working days missed due to sickness</t>
+  </si>
+  <si>
+    <t>https://www.gov.uk/government/collections/healthcare-associated-infections-hcai-guidance-data-and-analysis</t>
+  </si>
+  <si>
+    <t>number and rate per bed days (c-diff, surgical site, pneuomina, ecoli, klebsiella)</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>https://www.england.nhs.uk/fft/friends-and-family-test-data/; UKHF</t>
   </si>
 </sst>
 </file>
@@ -594,25 +600,25 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
         <v>3</v>
       </c>
       <c r="H1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" t="s">
         <v>29</v>
-      </c>
-      <c r="I1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.75">
@@ -623,13 +629,16 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>55</v>
       </c>
       <c r="G2" t="s">
         <v>6</v>
@@ -638,7 +647,7 @@
         <v>7</v>
       </c>
       <c r="I2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.75">
@@ -649,22 +658,25 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" t="s">
         <v>32</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="H3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.75">
@@ -675,14 +687,17 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
       </c>
+      <c r="F4" t="s">
+        <v>55</v>
+      </c>
       <c r="G4" t="s">
         <v>11</v>
       </c>
@@ -690,7 +705,7 @@
         <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.75">
@@ -701,14 +716,17 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
       </c>
+      <c r="F5" t="s">
+        <v>55</v>
+      </c>
       <c r="G5" t="s">
         <v>11</v>
       </c>
@@ -716,7 +734,7 @@
         <v>12</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.75">
@@ -724,16 +742,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
       </c>
       <c r="G6" t="s">
         <v>6</v>
@@ -742,7 +763,7 @@
         <v>14</v>
       </c>
       <c r="I6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.75">
@@ -753,14 +774,17 @@
         <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
       </c>
+      <c r="F7" t="s">
+        <v>55</v>
+      </c>
       <c r="G7" t="s">
         <v>11</v>
       </c>
@@ -768,7 +792,7 @@
         <v>12</v>
       </c>
       <c r="I7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.75">
@@ -779,14 +803,17 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
       </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
@@ -794,7 +821,7 @@
         <v>19</v>
       </c>
       <c r="I8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.75">
@@ -802,25 +829,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" t="s">
         <v>37</v>
       </c>
-      <c r="C9" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="H9" t="s">
         <v>40</v>
       </c>
-      <c r="G9" t="s">
-        <v>39</v>
-      </c>
-      <c r="H9" t="s">
-        <v>42</v>
-      </c>
       <c r="I9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.75">
@@ -831,22 +861,25 @@
         <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" t="s">
-        <v>21</v>
+        <v>34</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
       </c>
       <c r="G10" t="s">
         <v>6</v>
       </c>
       <c r="H10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.75">
@@ -854,25 +887,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C11" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>24</v>
+      <c r="F11" t="s">
+        <v>56</v>
       </c>
       <c r="G11" t="s">
         <v>6</v>
       </c>
       <c r="H11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.75">
@@ -880,25 +916,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>27</v>
+      <c r="F12" t="s">
+        <v>56</v>
       </c>
       <c r="G12" t="s">
         <v>6</v>
       </c>
       <c r="H12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -908,6 +947,9 @@
     <hyperlink ref="E6" r:id="rId2" xr:uid="{89902B8E-A5E0-4B1D-A9E2-7FBCFC60C961}"/>
     <hyperlink ref="E11" r:id="rId3" xr:uid="{6FD042B7-9CF5-405A-80F5-B7B20B69455A}"/>
     <hyperlink ref="E12" r:id="rId4" xr:uid="{EDDCA832-209B-4741-937D-6DCB9F831006}"/>
+    <hyperlink ref="E3" r:id="rId5" xr:uid="{D0229BA6-9FC3-4DD6-BB28-45BC00590C8E}"/>
+    <hyperlink ref="E2" r:id="rId6" xr:uid="{093F9F6B-7D9B-4638-9710-9A122C853D2C}"/>
+    <hyperlink ref="E10" r:id="rId7" xr:uid="{852A6D88-0B5D-4A26-9344-C8BA9FB447CB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Assign indicators to SL and AF to collect.
</commit_message>
<xml_diff>
--- a/indicator_summary.xlsx
+++ b/indicator_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FB09759-1EED-457B-8AA7-73BCE596F62C}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61846C26-14A0-4415-86FB-D631A3159E46}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="62">
   <si>
     <t>id</t>
   </si>
@@ -89,9 +89,6 @@
     <t>Occupancy levels</t>
   </si>
   <si>
-    <t>TBC, sitreps or KH03</t>
-  </si>
-  <si>
     <t>M/Q</t>
   </si>
   <si>
@@ -179,9 +176,6 @@
     <t>Waiting list / times</t>
   </si>
   <si>
-    <t>incomplete pathways, number and mean time</t>
-  </si>
-  <si>
     <t>ratio of observed to expected deaths</t>
   </si>
   <si>
@@ -191,9 +185,6 @@
     <t>WTE number and rate per bed days</t>
   </si>
   <si>
-    <t>TBC. Maybe % vacancies?</t>
-  </si>
-  <si>
     <t>% working days missed due to sickness</t>
   </si>
   <si>
@@ -210,6 +201,27 @@
   </si>
   <si>
     <t>https://www.england.nhs.uk/fft/friends-and-family-test-data/; UKHF</t>
+  </si>
+  <si>
+    <t>resp</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>SL</t>
+  </si>
+  <si>
+    <t>Sitreps and KH03 (https://www.england.nhs.uk/statistics/statistical-work-areas/bed-availability-and-occupancy/)</t>
+  </si>
+  <si>
+    <t>TBC. Maybe % vacancies, nursing?</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>incomplete pathways, number and median wait time</t>
   </si>
 </sst>
 </file>
@@ -260,9 +272,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -578,366 +598,404 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E08EDD4-E7EE-4C3F-874F-C71715322AB2}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="2.76953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.58984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="114.58984375" customWidth="1"/>
-    <col min="6" max="6" width="15.04296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.04296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.76953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.2265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="44.08984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.6796875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.04296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.04296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.75">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="I9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="H10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G3" t="s">
+    </row>
+    <row r="12" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" t="s">
-        <v>56</v>
-      </c>
-      <c r="G6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="H12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="J12" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="F10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" t="s">
-        <v>6</v>
-      </c>
-      <c r="H10" t="s">
-        <v>21</v>
-      </c>
-      <c r="I10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" t="s">
-        <v>56</v>
-      </c>
-      <c r="G11" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.75">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F12" t="s">
-        <v>56</v>
-      </c>
-      <c r="G12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H12" t="s">
-        <v>27</v>
-      </c>
-      <c r="I12" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding date filter to shmi query
</commit_message>
<xml_diff>
--- a/indicator_summary.xlsx
+++ b/indicator_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/anya_ferguson_mlcsu_nhs_uk/Documents/Desktop/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="53" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61846C26-14A0-4415-86FB-D631A3159E46}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -302,9 +302,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -342,7 +342,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -448,7 +448,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -590,7 +590,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -599,22 +599,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E08EDD4-E7EE-4C3F-874F-C71715322AB2}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.76953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.2265625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1796875" style="1" customWidth="1"/>
     <col min="3" max="3" width="44.08984375" style="1" customWidth="1"/>
     <col min="4" max="4" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.6796875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.04296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.08984375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.04296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="4.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -646,7 +646,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -678,7 +678,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -710,7 +710,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -742,7 +742,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -774,7 +774,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -806,7 +806,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -838,7 +838,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -870,7 +870,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -902,7 +902,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -934,7 +934,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -966,7 +966,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Changes to indicator descriptions table (excel file, to be called when complete), additional refs and added introduction section text.
</commit_message>
<xml_diff>
--- a/indicator_summary.xlsx
+++ b/indicator_summary.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7A52C29-6A60-4159-91A2-1C4A980654B7}"/>
+  <xr:revisionPtr revIDLastSave="142" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B6B5FAE-0090-46A8-959F-7BD69199A89D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="10620" windowWidth="29040" windowHeight="15840" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" activeTab="1" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="og" sheetId="1" r:id="rId1"/>
+    <sheet name="new" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="103">
   <si>
     <t>id</t>
   </si>
@@ -246,13 +247,112 @@
   </si>
   <si>
     <t>genericise, check codes, monthly etc…</t>
+  </si>
+  <si>
+    <t>Hospital deaths</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>derivation_notes</t>
+  </si>
+  <si>
+    <t>Healthcare Associated Infections - clostridium difficile</t>
+  </si>
+  <si>
+    <t>Falls and injuries</t>
+  </si>
+  <si>
+    <t>Waiting time</t>
+  </si>
+  <si>
+    <t>Bed occupancy</t>
+  </si>
+  <si>
+    <t>Cleaning costs</t>
+  </si>
+  <si>
+    <t>Staff sickness</t>
+  </si>
+  <si>
+    <t>Staff experience</t>
+  </si>
+  <si>
+    <t>Ordinary inpatient only. Stillbirth excluded. NHS providers only.</t>
+  </si>
+  <si>
+    <t>Distinct spells where episode order in spell &gt; 1 AND ICD-10 code in (W01, W03-W08, W18-W19, S0-S9, T0, T10-T14) where non present in first episode.</t>
+  </si>
+  <si>
+    <t>Rate of death per 1,000 discharges.</t>
+  </si>
+  <si>
+    <t>Mean length of stay</t>
+  </si>
+  <si>
+    <t>Cases per 10,000 bed days</t>
+  </si>
+  <si>
+    <t>Spells with fall as % of all spells</t>
+  </si>
+  <si>
+    <t>Median wait time in weeks</t>
+  </si>
+  <si>
+    <t>% available beds occupied overnight</t>
+  </si>
+  <si>
+    <t>Family and friends test, % positive scores (inpatient)</t>
+  </si>
+  <si>
+    <t>% available days taken off sick</t>
+  </si>
+  <si>
+    <t>% staff recommending the trust as place to work</t>
+  </si>
+  <si>
+    <t>Derived from SUS admitted patient care data (NCDR)</t>
+  </si>
+  <si>
+    <t>https://www.england.nhs.uk/statistics/statistical-work-areas/rtt-waiting-times</t>
+  </si>
+  <si>
+    <t>https://www.england.nhs.uk/statistics/statistical-work-areas/bed-availability-and-occupancy/</t>
+  </si>
+  <si>
+    <t>https://www.england.nhs.uk/fft/friends-and-family-test-data/</t>
+  </si>
+  <si>
+    <t>https://www.nhsstaffsurveys.com/results/</t>
+  </si>
+  <si>
+    <t>Ordinary inpatient only, deaths excluded, completed spells only, NHS providers only.</t>
+  </si>
+  <si>
+    <t>% of discharges with emergency readmission &lt; 30 days</t>
+  </si>
+  <si>
+    <t>Ordinary inpatient only, discharge method = 1 or 3</t>
+  </si>
+  <si>
+    <t>Bed days denominator derived from SUS APCE</t>
+  </si>
+  <si>
+    <t>Denominator TBC</t>
+  </si>
+  <si>
+    <t>Total cleaning costs (per denominator TBC)</t>
+  </si>
+  <si>
+    <t>rationale</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +370,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -296,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -306,6 +412,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -326,9 +445,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -366,7 +485,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -472,7 +591,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -614,7 +733,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -623,23 +742,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E08EDD4-E7EE-4C3F-874F-C71715322AB2}">
   <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.76953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.2265625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1796875" style="1" customWidth="1"/>
     <col min="3" max="3" width="44.08984375" style="1" customWidth="1"/>
     <col min="4" max="4" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.6796875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.04296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.08984375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.04296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="4.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.58984375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.54296875" style="1" customWidth="1"/>
     <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -674,7 +793,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -709,7 +828,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="59" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -744,7 +863,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -779,7 +898,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -814,7 +933,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -849,7 +968,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -884,7 +1003,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -919,7 +1038,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -954,7 +1073,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -989,7 +1108,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1024,7 +1143,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1072,4 +1191,260 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEB74C0B-FF78-4536-9B07-D64BF15FDFB9}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.36328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.90625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.90625" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="110.90625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E9" r:id="rId1" xr:uid="{5549AA0B-DE30-4035-A22C-ED9A90EFA7F6}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{2B35D968-8B42-486D-B18F-FEB48ADC7F3B}"/>
+    <hyperlink ref="E11" r:id="rId3" xr:uid="{B0BAA521-4C76-4410-8691-CC9F856C7502}"/>
+    <hyperlink ref="E3" r:id="rId4" xr:uid="{71810FEA-8EE9-4397-86AF-E2D56E6C7E9A}"/>
+    <hyperlink ref="E10" r:id="rId5" xr:uid="{C2E447C6-06F3-4BAB-9C2C-FA1D21DE4A32}"/>
+    <hyperlink ref="E8" r:id="rId6" xr:uid="{A7396356-E6C5-4A3E-90DC-CB8095646716}"/>
+    <hyperlink ref="E12" r:id="rId7" xr:uid="{1BB3A0B0-2C1F-4D1C-B187-54B47D9A40B5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Editing and adding staff turnover to indicator table
</commit_message>
<xml_diff>
--- a/indicator_summary.xlsx
+++ b/indicator_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="142" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B6B5FAE-0090-46A8-959F-7BD69199A89D}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F9D280C-56C3-408C-9BC8-2E1CE04CD9B2}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" activeTab="1" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="13800" activeTab="1" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
   </bookViews>
   <sheets>
     <sheet name="og" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="103">
   <si>
     <t>id</t>
   </si>
@@ -339,13 +339,13 @@
     <t>Bed days denominator derived from SUS APCE</t>
   </si>
   <si>
-    <t>Denominator TBC</t>
-  </si>
-  <si>
-    <t>Total cleaning costs (per denominator TBC)</t>
-  </si>
-  <si>
     <t>rationale</t>
+  </si>
+  <si>
+    <t>Total cleaning costs (£/sqm of occupied floor space)</t>
+  </si>
+  <si>
+    <t>% of staff leaving</t>
   </si>
 </sst>
 </file>
@@ -402,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -416,11 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -742,23 +738,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E08EDD4-E7EE-4C3F-874F-C71715322AB2}">
   <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.1796875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="44.08984375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.6328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="44.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.6640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.54296875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="1"/>
+    <col min="10" max="10" width="4.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5546875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -793,7 +789,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -828,7 +824,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -863,7 +859,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -898,7 +894,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -933,7 +929,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -968,7 +964,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1003,7 +999,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1038,7 +1034,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1073,7 +1069,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1108,7 +1104,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1143,7 +1139,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1195,19 +1191,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEB74C0B-FF78-4536-9B07-D64BF15FDFB9}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.36328125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.90625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.90625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="110.90625" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="54.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="5"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="110.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1223,14 +1218,14 @@
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" t="s">
         <v>72</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1243,14 +1238,14 @@
       <c r="D2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1263,14 +1258,14 @@
       <c r="D3" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1283,14 +1278,14 @@
       <c r="D4" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1303,14 +1298,14 @@
       <c r="D5" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>91</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1323,11 +1318,11 @@
       <c r="D6" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1340,14 +1335,14 @@
       <c r="D7" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="6" t="s">
         <v>91</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1360,11 +1355,11 @@
       <c r="D8" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1377,14 +1372,12 @@
       <c r="D9" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1397,11 +1390,11 @@
       <c r="D10" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1414,11 +1407,11 @@
       <c r="D11" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1426,12 +1419,29 @@
         <v>32</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1443,7 +1453,7 @@
     <hyperlink ref="E3" r:id="rId4" xr:uid="{71810FEA-8EE9-4397-86AF-E2D56E6C7E9A}"/>
     <hyperlink ref="E10" r:id="rId5" xr:uid="{C2E447C6-06F3-4BAB-9C2C-FA1D21DE4A32}"/>
     <hyperlink ref="E8" r:id="rId6" xr:uid="{A7396356-E6C5-4A3E-90DC-CB8095646716}"/>
-    <hyperlink ref="E12" r:id="rId7" xr:uid="{1BB3A0B0-2C1F-4D1C-B187-54B47D9A40B5}"/>
+    <hyperlink ref="E13" r:id="rId7" xr:uid="{1BB3A0B0-2C1F-4D1C-B187-54B47D9A40B5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add rationale to indicator summary table.
</commit_message>
<xml_diff>
--- a/indicator_summary.xlsx
+++ b/indicator_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F9D280C-56C3-408C-9BC8-2E1CE04CD9B2}"/>
+  <xr:revisionPtr revIDLastSave="179" documentId="8_{0A14007F-8643-4553-9B09-86BF0F47155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2EB9393-9F06-4202-992C-92CD865E53AE}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="13800" activeTab="1" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{ED844CE7-538F-42B8-9E21-F34E5658EA61}"/>
   </bookViews>
   <sheets>
     <sheet name="og" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="115">
   <si>
     <t>id</t>
   </si>
@@ -346,6 +346,42 @@
   </si>
   <si>
     <t>% of staff leaving</t>
+  </si>
+  <si>
+    <t>Patients could miss out on informal observations by both staff and other patients thus missing critical changes in symptoms. Whilst there is mixed evidence of SBR impacts on mortality, several studies have shown a significant increase in the general adult population.</t>
+  </si>
+  <si>
+    <t>Single bed rooms remove other patients as vectors for transmitting infectious pathogens. The WHO have concluded that single rooms reduce HCAI.</t>
+  </si>
+  <si>
+    <t>Single rooms with greater volume of equipment, more 'wet space' and lower levels of casual observation may increase the risk of patient falls and injuries.</t>
+  </si>
+  <si>
+    <t>Privacy and improved sleep can lead to quicker recovery and therefore reduced length of stay in single bed rooms for some patients. Higher-quality research suggests shorter hospital stays are likely.</t>
+  </si>
+  <si>
+    <t>Logically, shorter length of stay and greater flexibility of bed stock (occupancy) mean that waiting lists and times are likely to reduce all other things equal.</t>
+  </si>
+  <si>
+    <t>Evidence is scarce for the direction and scale of impacts on readmission with some studies citing an increase others a decrease for patients of different types.</t>
+  </si>
+  <si>
+    <t>Single bed rooms are thought to offer  more flexibility in use of bed stock - single rooms can be closed due to infectious incidents for example rather than whole wards making management of emergency cases less impactful.</t>
+  </si>
+  <si>
+    <t>Single ensuite rooms mean both more wet areas to clean and more movement of equipment and personnel between rooms. Evidence suggests day-to-day management costs of single beds is greater.</t>
+  </si>
+  <si>
+    <t>Some patients prefer the privacy and lack of disturbance from single rooms whilst others prefer the social interaction of shared space. There is mixed evidence around patient satisfaction resulting from switch to single bed rooms.</t>
+  </si>
+  <si>
+    <t>Recent studies suggest that staff have strong reservations about single rooms related to stress and personal safety.</t>
+  </si>
+  <si>
+    <t>Fewer multi-patient exposures and additional infection control steps may lead to decreased staff absence from illness.</t>
+  </si>
+  <si>
+    <t>Linked to staff experience, the rate of staff leavers may increase with increased disatisfaction at work.</t>
   </si>
 </sst>
 </file>
@@ -402,7 +438,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -414,13 +450,16 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -738,23 +777,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E08EDD4-E7EE-4C3F-874F-C71715322AB2}">
   <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.21875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1796875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="44.08984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.6328125" style="1" customWidth="1"/>
     <col min="6" max="6" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5546875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.77734375" style="1"/>
+    <col min="10" max="10" width="4.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.54296875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -789,7 +828,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -824,7 +863,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -859,7 +898,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -894,7 +933,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -929,7 +968,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -964,7 +1003,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -999,7 +1038,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1034,7 +1073,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1069,7 +1108,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1104,7 +1143,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1139,7 +1178,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1192,17 +1231,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEB74C0B-FF78-4536-9B07-D64BF15FDFB9}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="110.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="54.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.36328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.1796875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="28.81640625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="110.90625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.36328125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="36.7265625" style="7" customWidth="1"/>
+    <col min="8" max="16384" width="8.81640625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1218,14 +1259,14 @@
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>72</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1238,14 +1279,17 @@
       <c r="D2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>91</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1258,14 +1302,17 @@
       <c r="D3" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>49</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G3" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1278,14 +1325,17 @@
       <c r="D4" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G4" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1298,14 +1348,17 @@
       <c r="D5" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>91</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G5" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1318,11 +1371,15 @@
       <c r="D6" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F6" s="4"/>
+      <c r="G6" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1335,14 +1392,17 @@
       <c r="D7" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>91</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G7" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1355,11 +1415,15 @@
       <c r="D8" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F8" s="4"/>
+      <c r="G8" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1372,12 +1436,15 @@
       <c r="D9" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G9" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1390,11 +1457,15 @@
       <c r="D10" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F10" s="4"/>
+      <c r="G10" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1407,11 +1478,15 @@
       <c r="D11" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F11" s="4"/>
+      <c r="G11" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1424,11 +1499,15 @@
       <c r="D12" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F12" s="4"/>
+      <c r="G12" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -1441,8 +1520,12 @@
       <c r="D13" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>95</v>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>